<commit_message>
almost working CREATE benchmark
</commit_message>
<xml_diff>
--- a/tests/CREATE_force_measurement/input_template.xlsx
+++ b/tests/CREATE_force_measurement/input_template.xlsx
@@ -225,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -243,12 +243,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -559,20 +553,20 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="14.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="14.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -622,7 +616,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -645,7 +639,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
@@ -682,7 +676,7 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
@@ -723,7 +717,7 @@
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="20.14785714285714" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -768,130 +762,130 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="6">
-        <v>1</v>
-      </c>
-      <c r="B2" s="8">
-        <v>1</v>
-      </c>
-      <c r="C2" s="8">
-        <v>1</v>
-      </c>
-      <c r="D2" s="8">
-        <v>1</v>
-      </c>
-      <c r="E2" s="8">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2">
         <v>3e-7</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="2">
         <v>3e-7</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="2">
         <v>3e-7</v>
       </c>
-      <c r="H2" s="8">
-        <v>0</v>
-      </c>
-      <c r="I2" s="8">
-        <v>0</v>
-      </c>
-      <c r="J2" s="8">
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="8">
-        <v>1</v>
-      </c>
-      <c r="C3" s="8">
-        <v>1</v>
-      </c>
-      <c r="D3" s="8">
-        <v>1</v>
-      </c>
-      <c r="E3" s="8">
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
         <v>1.09e-7</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="2">
         <v>1.09e-7</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="2">
         <v>1.09e-7</v>
       </c>
-      <c r="H3" s="8">
-        <v>0</v>
-      </c>
-      <c r="I3" s="8">
-        <v>0</v>
-      </c>
-      <c r="J3" s="8">
+      <c r="H3" s="2">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="6">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="8">
-        <v>1</v>
-      </c>
-      <c r="C4" s="8">
-        <v>1</v>
-      </c>
-      <c r="D4" s="8">
-        <v>1</v>
-      </c>
-      <c r="E4" s="8">
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2">
         <v>10</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="2">
         <v>10</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="2">
         <v>10</v>
       </c>
-      <c r="H4" s="8">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0</v>
-      </c>
-      <c r="J4" s="8">
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>10</v>
       </c>
-      <c r="B5" s="8">
-        <v>1</v>
-      </c>
-      <c r="C5" s="8">
-        <v>1</v>
-      </c>
-      <c r="D5" s="8">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8">
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2">
         <v>2.13e-8</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="2">
         <v>2.13e-8</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="2">
         <v>2.13e-8</v>
       </c>
-      <c r="H5" s="8">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8">
-        <v>0</v>
-      </c>
-      <c r="J5" s="8">
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -940,26 +934,26 @@
   <dimension ref="A1:T6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="21.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="19.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="21.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="19.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -1025,250 +1019,250 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="6">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>127</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="6">
-        <v>0</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0</v>
-      </c>
-      <c r="J2" s="6">
+      <c r="F2" s="3">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3">
         <v>1.144</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="3">
         <v>2</v>
       </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2" s="3">
+        <v>0</v>
+      </c>
+      <c r="N2" s="3">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3">
+        <v>0</v>
+      </c>
+      <c r="P2" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>0</v>
+      </c>
+      <c r="R2" s="3">
+        <v>0</v>
+      </c>
+      <c r="S2" s="3">
+        <v>0</v>
+      </c>
+      <c r="T2" s="3">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="6">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6" t="s">
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>127</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="6">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>1</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="6">
+      <c r="F3" s="3">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
         <v>1.144</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>2</v>
       </c>
-      <c r="L3" s="6">
-        <v>0</v>
-      </c>
-      <c r="M3" s="6">
-        <v>0</v>
-      </c>
-      <c r="N3" s="6">
-        <v>0</v>
-      </c>
-      <c r="O3" s="6">
-        <v>0</v>
-      </c>
-      <c r="P3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="6">
-        <v>0</v>
-      </c>
-      <c r="R3" s="6">
-        <v>0</v>
-      </c>
-      <c r="S3" s="6">
-        <v>0</v>
-      </c>
-      <c r="T3" s="6">
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3">
+        <v>0</v>
+      </c>
+      <c r="P3" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>0</v>
+      </c>
+      <c r="R3" s="3">
+        <v>0</v>
+      </c>
+      <c r="S3" s="3">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="6">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="6">
-        <v>1</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>127</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
         <v>1.144</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>2</v>
       </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="6">
-        <v>0</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6">
-        <v>0</v>
-      </c>
-      <c r="P4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="6">
-        <v>0</v>
-      </c>
-      <c r="R4" s="6">
-        <v>0</v>
-      </c>
-      <c r="S4" s="6">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6">
+      <c r="L4" s="3">
+        <v>0</v>
+      </c>
+      <c r="M4" s="3">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3">
+        <v>0</v>
+      </c>
+      <c r="P4" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>0</v>
+      </c>
+      <c r="R4" s="3">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3">
+        <v>0</v>
+      </c>
+      <c r="T4" s="3">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="6">
-        <v>1</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>127</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6">
-        <v>0</v>
-      </c>
-      <c r="J5" s="6">
+      <c r="F5" s="3">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3">
+        <v>1</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3">
         <v>1.144</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>2</v>
       </c>
-      <c r="L5" s="6">
-        <v>0</v>
-      </c>
-      <c r="M5" s="6">
-        <v>0</v>
-      </c>
-      <c r="N5" s="6">
-        <v>0</v>
-      </c>
-      <c r="O5" s="6">
-        <v>0</v>
-      </c>
-      <c r="P5" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="6">
-        <v>0</v>
-      </c>
-      <c r="R5" s="6">
-        <v>0</v>
-      </c>
-      <c r="S5" s="6">
-        <v>0</v>
-      </c>
-      <c r="T5" s="6">
+      <c r="L5" s="3">
+        <v>0</v>
+      </c>
+      <c r="M5" s="3">
+        <v>0</v>
+      </c>
+      <c r="N5" s="3">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3">
+        <v>0</v>
+      </c>
+      <c r="P5" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>0</v>
+      </c>
+      <c r="R5" s="3">
+        <v>0</v>
+      </c>
+      <c r="S5" s="3">
+        <v>0</v>
+      </c>
+      <c r="T5" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>